<commit_message>
Rev D: align full PCB lot order and procurement summary
</commit_message>
<xml_diff>
--- a/releases/evt-pre-20/2026-09-30-rev-d/Заказ_плат_и_монтаж/00_Условия_передачи/BOM_плат_для_монтажа.xlsx
+++ b/releases/evt-pre-20/2026-09-30-rev-d/Заказ_плат_и_монтаж/00_Условия_передачи/BOM_плат_для_монтажа.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB-PWR BOM" sheetId="1" r:id="Rbf71a3b4f4b14778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB-PWR DNP" sheetId="2" r:id="R503dcbdc3f0144e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB-MIC BOM" sheetId="3" r:id="R6e1d367e3e2d4808"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB-MAIN BOM" sheetId="4" r:id="R79aa01736290445c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="5" r:id="R4e421414b9864b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB-PWR BOM" sheetId="1" r:id="Rf672952b1c7b4919"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB-PWR DNP" sheetId="2" r:id="R07f1b1dca931430e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB-MIC BOM" sheetId="3" r:id="Rc2291683610d4e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB-MAIN BOM" sheetId="4" r:id="Rec5f936d12dc4de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="5" r:id="R26cd351c6ac743c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7403,7 +7403,7 @@
         <x:v>Монтаж / Assembly</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Первый образец / First article</x:v>
+        <x:v>Выборка после партии / Post-lot sample</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
         <x:v>Статус / Status</x:v>
@@ -7414,7 +7414,7 @@
         <x:v>PCB-MAIN</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
-        <x:v>22 PCBA</x:v>
+        <x:v>22 PCBA, one full lot</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
         <x:v>PCB-MAIN BOM, DNP, off-board</x:v>
@@ -7423,10 +7423,10 @@
         <x:v>227 PCBA placements; 15 DNP; U12 off-board</x:v>
       </x:c>
       <x:c r="E3" s="5" t="str">
-        <x:v>2 изделия / units</x:v>
+        <x:v>2 units after build</x:v>
       </x:c>
       <x:c r="F3" s="5" t="str">
-        <x:v>DRC 0; unconnected 0; ERC 0; fab DFM and stack confirmation</x:v>
+        <x:v>No pause; DFM, stack and 76 POFV before panel</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="31" customHeight="1">
@@ -7434,7 +7434,7 @@
         <x:v>PCB-PWR</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>22 PCBA</x:v>
+        <x:v>22 PCBA, one full lot</x:v>
       </x:c>
       <x:c r="C4" s="5" t="str">
         <x:v>44 fitted; 5 DNP; 3 copper net ties</x:v>
@@ -7443,10 +7443,10 @@
         <x:v>Use position CSV and RU/EN assembly drawing</x:v>
       </x:c>
       <x:c r="E4" s="5" t="str">
-        <x:v>2 изделия / units</x:v>
+        <x:v>2 units after build</x:v>
       </x:c>
       <x:c r="F4" s="5" t="str">
-        <x:v>Order authorized; fab DFM and stack confirmation</x:v>
+        <x:v>No pause; fab DFM and stack confirmation</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="31" customHeight="1">
@@ -7454,7 +7454,7 @@
         <x:v>PCB-MIC Rev B</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>80 PCBA</x:v>
+        <x:v>80 PCBA, one full lot</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
         <x:v>4 fitted per board</x:v>
@@ -7463,10 +7463,10 @@
         <x:v>Acoustic port Ø0.8 NPTH; MK1 stencil controlled</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
-        <x:v>1 board/panel → remaining 79</x:v>
+        <x:v>1 board/panel after build</x:v>
       </x:c>
       <x:c r="F5" s="5" t="str">
-        <x:v>Review B ACCEPT CONTROLLED FIRST ARTICLE</x:v>
+        <x:v>Customer schedule supersedes Review B pause only</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>